<commit_message>
test(article-creation): Add E2E tests for article creation
Refs: #8
</commit_message>
<xml_diff>
--- a/docs/features.xlsx
+++ b/docs/features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t xml:space="preserve">Feature</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🟠 Medium</t>
   </si>
 </sst>
 </file>
@@ -169,7 +175,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.86"/>
@@ -213,6 +219,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[#8] E2E tests for article creation (#12)
* test(article-creation): Add E2E tests for article creation

Refs: #8

* feat(e2e): Implement global setup and teardown for authentication in tests

* refactor(api): Update API URL handling and improve regex escaping in utilities

Refs: #8

---------

Co-authored-by: idembele70 <idembele70@gmail>
</commit_message>
<xml_diff>
--- a/docs/features.xlsx
+++ b/docs/features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t xml:space="preserve">Feature</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🟠 Medium</t>
   </si>
 </sst>
 </file>
@@ -169,7 +175,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.86"/>
@@ -213,6 +219,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>